<commit_message>
tweaked data input for easyrsei
</commit_message>
<xml_diff>
--- a/easyrsei_2022_air.xlsx
+++ b/easyrsei_2022_air.xlsx
@@ -34,6 +34,18 @@
     <t>TRI Pounds</t>
   </si>
   <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>WABTEC COMPONENTS LLC FORMERLY THERMAL TRANSFER CORP</t>
+  </si>
+  <si>
+    <t>50 N LINDEN ST</t>
+  </si>
+  <si>
+    <t>DUQUESNE, PA</t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
@@ -46,6 +58,75 @@
     <t>CLAIRTON, PA</t>
   </si>
   <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>PPG INDUSTRIESINC-SPRINGDALE COMPLEX</t>
+  </si>
+  <si>
+    <t>125 COLFAX ST</t>
+  </si>
+  <si>
+    <t>SPRINGDALE, PA</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>UNIVERSAL STAINLESS &amp; ALLOY PRODUCTS INC</t>
+  </si>
+  <si>
+    <t>600 MAYER ST</t>
+  </si>
+  <si>
+    <t>BRIDGEVILLE, PA</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>TMS INTERNATIONAL LLC</t>
+  </si>
+  <si>
+    <t>1300 BRADDOCK AVE</t>
+  </si>
+  <si>
+    <t>BRADDOCK, PA</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>MCCONWAY &amp; TORLEY LLC PLT 1801</t>
+  </si>
+  <si>
+    <t>109 48TH ST</t>
+  </si>
+  <si>
+    <t>PITTSBURGH, PA</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>ATI FLAT ROLLED PRODUCTS HOLDINGS LLC</t>
+  </si>
+  <si>
+    <t>100 RIVER RD</t>
+  </si>
+  <si>
+    <t>BRACKENRIDGE, PA</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>NEVILLE CHEMICAL CO</t>
+  </si>
+  <si>
+    <t>2800 NEVILLE RD</t>
+  </si>
+  <si>
     <t>9</t>
   </si>
   <si>
@@ -55,7 +136,67 @@
     <t>BRADDOCK AVE &amp; 13TH ST</t>
   </si>
   <si>
-    <t>BRADDOCK, PA</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>ATI POWDER METALS - OAKDALE</t>
+  </si>
+  <si>
+    <t>1001 ROBB HILL RD</t>
+  </si>
+  <si>
+    <t>OAKDALE, PA</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>CURTISS WRIGHT ELECTRO MECH CORP</t>
+  </si>
+  <si>
+    <t>1000 WRIGHT WAY</t>
+  </si>
+  <si>
+    <t>CHESWICK, PA</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>CHASE CORP - PITTSBURGH</t>
+  </si>
+  <si>
+    <t>201 ZETA DRIVE</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>HOLTEC MANUFACTURING</t>
+  </si>
+  <si>
+    <t>750 BRADDOCK AVE</t>
+  </si>
+  <si>
+    <t>EAST PITTSBURGH, PA</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>INEOS COMPOSITES US LLC</t>
+  </si>
+  <si>
+    <t>2650 NEVILLE RD</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>MATTHEWS INTERNATIONAL CORP</t>
+  </si>
+  <si>
+    <t>1315 W LIBERTY AVE</t>
   </si>
   <si>
     <t>16</t>
@@ -70,16 +211,55 @@
     <t>LEETSDALE, PA</t>
   </si>
   <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>ATI FLAT ROLLED PRODUCTS HOLDINGS LLC</t>
-  </si>
-  <si>
-    <t>100 RIVER RD</t>
-  </si>
-  <si>
-    <t>BRACKENRIDGE, PA</t>
+    <t>17</t>
+  </si>
+  <si>
+    <t>USS MON VALLEY WORKS - IRVIN PLANT</t>
+  </si>
+  <si>
+    <t>CAMP HOLLOW RD</t>
+  </si>
+  <si>
+    <t>WEST MIFFLIN, PA</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>CHESWICK PLANT ENVIRONMENTAL REDEVELOPMENT GROUP LLC</t>
+  </si>
+  <si>
+    <t>PITTSBURGH &amp; PORTER ST</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>SUPERIOR FORGE &amp; STEEL CORP</t>
+  </si>
+  <si>
+    <t>1101 MURIEL ST</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>TECH MET INC.</t>
+  </si>
+  <si>
+    <t>15 ALLEGHENY SQUARE</t>
+  </si>
+  <si>
+    <t>GLASSPORT, PA</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>CALGON CARBON CORP NEVILLE ISLAND PLANT</t>
+  </si>
+  <si>
+    <t>200 NEVILLE RD</t>
   </si>
   <si>
     <t>22</t>
@@ -94,85 +274,103 @@
     <t>JEFFERSON HILLS, PA</t>
   </si>
   <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>PPG INDUSTRIESINC-SPRINGDALE COMPLEX</t>
-  </si>
-  <si>
-    <t>125 COLFAX ST</t>
-  </si>
-  <si>
-    <t>SPRINGDALE, PA</t>
-  </si>
-  <si>
-    <t>6</t>
-  </si>
-  <si>
-    <t>MCCONWAY &amp; TORLEY LLC PLT 1801</t>
-  </si>
-  <si>
-    <t>109 48TH ST</t>
-  </si>
-  <si>
-    <t>PITTSBURGH, PA</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>UNIVERSAL STAINLESS &amp; ALLOY PRODUCTS INC</t>
-  </si>
-  <si>
-    <t>600 MAYER ST</t>
-  </si>
-  <si>
-    <t>BRIDGEVILLE, PA</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>HOLTEC MANUFACTURING</t>
-  </si>
-  <si>
-    <t>750 BRADDOCK AVE</t>
-  </si>
-  <si>
-    <t>EAST PITTSBURGH, PA</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>MATTHEWS INTERNATIONAL CORP</t>
-  </si>
-  <si>
-    <t>1315 W LIBERTY AVE</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>WABTEC COMPONENTS LLC FORMERLY THERMAL TRANSFER CORP</t>
-  </si>
-  <si>
-    <t>50 N LINDEN ST</t>
-  </si>
-  <si>
-    <t>DUQUESNE, PA</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>USS MON VALLEY WORKS - IRVIN PLANT</t>
-  </si>
-  <si>
-    <t>CAMP HOLLOW RD</t>
-  </si>
-  <si>
-    <t>WEST MIFFLIN, PA</t>
+    <t>23</t>
+  </si>
+  <si>
+    <t>SHERWIN-WILLIAMS CO</t>
+  </si>
+  <si>
+    <t>2000 WESTHALL ST</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>KOPP GLASS INC</t>
+  </si>
+  <si>
+    <t>2108 PALMER ST</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>NORTHEAST PAVING BRIDGEVILLE PLANT</t>
+  </si>
+  <si>
+    <t>2 PRESTLEY ROAD</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>MARATHON PETROLEUM CO - FLOREFFE PA ASPHALT TERMINAL</t>
+  </si>
+  <si>
+    <t>1100 GLASS HOUSE RD</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>ALLEGHENY PETROLEUM PRODUCTS CO</t>
+  </si>
+  <si>
+    <t>999 AIRBRAKE AVE</t>
+  </si>
+  <si>
+    <t>WILMERDING, PA</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>LIBERTY PULTRUSIONS</t>
+  </si>
+  <si>
+    <t>1575 LEBANON SCHOOL RD</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>CHASE CORP-PITTSBURGH</t>
+  </si>
+  <si>
+    <t>128 FIRST ST</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>EPIC METALS CORP</t>
+  </si>
+  <si>
+    <t>11 TALBOT AVE</t>
+  </si>
+  <si>
+    <t>RANKIN, PA</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>STEEL DYNAMICS INC. - TECHS DIV - METALTECH PLANT</t>
+  </si>
+  <si>
+    <t>2400 2ND AVE</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>ASCENT TUBULAR PRODUCTS</t>
+  </si>
+  <si>
+    <t>1001 E WATERFRONT DR</t>
+  </si>
+  <si>
+    <t>MUNHALL, PA</t>
   </si>
   <si>
     <t>33</t>
@@ -184,6 +382,48 @@
     <t>3419 SMALLMAN ST</t>
   </si>
   <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>UNIVAR SOLUTIONS USA INC. - BUNOLA BRANCH</t>
+  </si>
+  <si>
+    <t>328 BUNOLA RIVER RD</t>
+  </si>
+  <si>
+    <t>BUNOLA, PA</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>BPI INC-MCKEES ROCKS PA PLANT</t>
+  </si>
+  <si>
+    <t>149 NICHOL AVE</t>
+  </si>
+  <si>
+    <t>MC KEES ROCKS, PA</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>LAFARGE - DUQUESNE SLAG</t>
+  </si>
+  <si>
+    <t>4810 BUTTERMILK HOLLOW ROAD</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>STEEL DYNAMICS INC. - TECHS DIV - GALVTECH PLANT</t>
+  </si>
+  <si>
+    <t>300 MIFFLIN RD</t>
+  </si>
+  <si>
     <t>38</t>
   </si>
   <si>
@@ -196,43 +436,13 @@
     <t>MONROEVILLE, PA</t>
   </si>
   <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>CALGON CARBON CORP NEVILLE ISLAND PLANT</t>
-  </si>
-  <si>
-    <t>200 NEVILLE RD</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>TECH MET INC.</t>
-  </si>
-  <si>
-    <t>15 ALLEGHENY SQUARE</t>
-  </si>
-  <si>
-    <t>GLASSPORT, PA</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>CHESWICK PLANT ENVIRONMENTAL REDEVELOPMENT GROUP LLC</t>
-  </si>
-  <si>
-    <t>PITTSBURGH &amp; PORTER ST</t>
-  </si>
-  <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>NEVILLE CHEMICAL CO</t>
-  </si>
-  <si>
-    <t>2800 NEVILLE RD</t>
+    <t>39</t>
+  </si>
+  <si>
+    <t>PITTSBURGH ELECTRICAL INSULATION</t>
+  </si>
+  <si>
+    <t>800 MARTHA ST</t>
   </si>
   <si>
     <t>40</t>
@@ -244,177 +454,6 @@
     <t>650 NOBLE DR</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>CHASE CORP - PITTSBURGH</t>
-  </si>
-  <si>
-    <t>201 ZETA DRIVE</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>INEOS COMPOSITES US LLC</t>
-  </si>
-  <si>
-    <t>2650 NEVILLE RD</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>LIBERTY PULTRUSIONS</t>
-  </si>
-  <si>
-    <t>1575 LEBANON SCHOOL RD</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>SHERWIN-WILLIAMS CO</t>
-  </si>
-  <si>
-    <t>2000 WESTHALL ST</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>ASCENT TUBULAR PRODUCTS</t>
-  </si>
-  <si>
-    <t>1001 E WATERFRONT DR</t>
-  </si>
-  <si>
-    <t>MUNHALL, PA</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>TMS INTERNATIONAL LLC</t>
-  </si>
-  <si>
-    <t>1300 BRADDOCK AVE</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>KOPP GLASS INC</t>
-  </si>
-  <si>
-    <t>2108 PALMER ST</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>ATI POWDER METALS - OAKDALE</t>
-  </si>
-  <si>
-    <t>1001 ROBB HILL RD</t>
-  </si>
-  <si>
-    <t>OAKDALE, PA</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>SUPERIOR FORGE &amp; STEEL CORP</t>
-  </si>
-  <si>
-    <t>1101 MURIEL ST</t>
-  </si>
-  <si>
-    <t>27</t>
-  </si>
-  <si>
-    <t>ALLEGHENY PETROLEUM PRODUCTS CO</t>
-  </si>
-  <si>
-    <t>999 AIRBRAKE AVE</t>
-  </si>
-  <si>
-    <t>WILMERDING, PA</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>CURTISS WRIGHT ELECTRO MECH CORP</t>
-  </si>
-  <si>
-    <t>1000 WRIGHT WAY</t>
-  </si>
-  <si>
-    <t>CHESWICK, PA</t>
-  </si>
-  <si>
-    <t>29</t>
-  </si>
-  <si>
-    <t>CHASE CORP-PITTSBURGH</t>
-  </si>
-  <si>
-    <t>128 FIRST ST</t>
-  </si>
-  <si>
-    <t>34</t>
-  </si>
-  <si>
-    <t>UNIVAR SOLUTIONS USA INC. - BUNOLA BRANCH</t>
-  </si>
-  <si>
-    <t>328 BUNOLA RIVER RD</t>
-  </si>
-  <si>
-    <t>BUNOLA, PA</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>EPIC METALS CORP</t>
-  </si>
-  <si>
-    <t>11 TALBOT AVE</t>
-  </si>
-  <si>
-    <t>RANKIN, PA</t>
-  </si>
-  <si>
-    <t>39</t>
-  </si>
-  <si>
-    <t>PITTSBURGH ELECTRICAL INSULATION</t>
-  </si>
-  <si>
-    <t>800 MARTHA ST</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>STEEL DYNAMICS INC. - TECHS DIV - METALTECH PLANT</t>
-  </si>
-  <si>
-    <t>2400 2ND AVE</t>
-  </si>
-  <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>STEEL DYNAMICS INC. - TECHS DIV - GALVTECH PLANT</t>
-  </si>
-  <si>
-    <t>300 MIFFLIN RD</t>
-  </si>
-  <si>
     <t>41</t>
   </si>
   <si>
@@ -422,45 +461,6 @@
   </si>
   <si>
     <t>148 NICHOL AVE - MRIE BLDG 162/163/164</t>
-  </si>
-  <si>
-    <t>MC KEES ROCKS, PA</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>MARATHON PETROLEUM CO - FLOREFFE PA ASPHALT TERMINAL</t>
-  </si>
-  <si>
-    <t>1100 GLASS HOUSE RD</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>NORTHEAST PAVING BRIDGEVILLE PLANT</t>
-  </si>
-  <si>
-    <t>2 PRESTLEY ROAD</t>
-  </si>
-  <si>
-    <t>36</t>
-  </si>
-  <si>
-    <t>LAFARGE - DUQUESNE SLAG</t>
-  </si>
-  <si>
-    <t>4810 BUTTERMILK HOLLOW ROAD</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>BPI INC-MCKEES ROCKS PA PLANT</t>
-  </si>
-  <si>
-    <t>149 NICHOL AVE</t>
   </si>
 </sst>
 </file>
@@ -841,10 +841,10 @@
         <v>9</v>
       </c>
       <c r="E2" s="1">
-        <v>83152.96620744601</v>
+        <v>250145.632729</v>
       </c>
       <c r="F2" s="1">
-        <v>9251497.6</v>
+        <v>219025</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -861,10 +861,10 @@
         <v>13</v>
       </c>
       <c r="E3" s="1">
-        <v>5536.45606</v>
+        <v>83152.96620744601</v>
       </c>
       <c r="F3" s="1">
-        <v>3311954.97</v>
+        <v>9251497.6</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -881,10 +881,10 @@
         <v>17</v>
       </c>
       <c r="E4" s="1">
-        <v>745.2152</v>
+        <v>77704.92790530247</v>
       </c>
       <c r="F4" s="1">
-        <v>2682415.3</v>
+        <v>759739.4739999999</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -901,10 +901,10 @@
         <v>21</v>
       </c>
       <c r="E5" s="1">
-        <v>12838.63171092</v>
+        <v>47409.30794400001</v>
       </c>
       <c r="F5" s="1">
-        <v>2364990.7</v>
+        <v>338413</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -921,10 +921,10 @@
         <v>25</v>
       </c>
       <c r="E6" s="1">
-        <v>32.29878160000001</v>
+        <v>36569.9404315</v>
       </c>
       <c r="F6" s="1">
-        <v>1879081.3</v>
+        <v>21076.455</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -941,10 +941,10 @@
         <v>29</v>
       </c>
       <c r="E7" s="1">
-        <v>77704.92790530247</v>
+        <v>12867.228911</v>
       </c>
       <c r="F7" s="1">
-        <v>759739.4740000003</v>
+        <v>501004</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -961,10 +961,10 @@
         <v>33</v>
       </c>
       <c r="E8" s="1">
-        <v>12867.228911</v>
+        <v>12838.63171092</v>
       </c>
       <c r="F8" s="1">
-        <v>501004</v>
+        <v>2364990.7</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -978,253 +978,253 @@
         <v>36</v>
       </c>
       <c r="D9" t="s">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="E9" s="1">
-        <v>47409.30794400001</v>
+        <v>7843.502919093998</v>
       </c>
       <c r="F9" s="1">
-        <v>338413</v>
+        <v>35155</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" t="s">
         <v>38</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>39</v>
       </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
       <c r="D10" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="E10" s="1">
-        <v>1750.380808</v>
+        <v>5536.45606</v>
       </c>
       <c r="F10" s="1">
-        <v>282837.304</v>
+        <v>3311954.97</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" t="s">
         <v>42</v>
       </c>
-      <c r="B11" t="s">
+      <c r="D11" t="s">
         <v>43</v>
       </c>
-      <c r="C11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" t="s">
-        <v>33</v>
-      </c>
       <c r="E11" s="1">
-        <v>1455.59946</v>
+        <v>3217.5016</v>
       </c>
       <c r="F11" s="1">
-        <v>276764</v>
+        <v>7799.26</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" t="s">
         <v>45</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>46</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>47</v>
       </c>
-      <c r="D12" t="s">
-        <v>48</v>
-      </c>
       <c r="E12" s="1">
-        <v>250145.632729</v>
+        <v>2285.37</v>
       </c>
       <c r="F12" s="1">
-        <v>219025</v>
+        <v>2221.03</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B13" t="s">
         <v>49</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>50</v>
       </c>
-      <c r="C13" t="s">
-        <v>51</v>
-      </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="E13" s="1">
-        <v>552.6938761</v>
+        <v>1992.54224118</v>
       </c>
       <c r="F13" s="1">
-        <v>166807.34</v>
+        <v>28260.55</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" t="s">
         <v>53</v>
       </c>
-      <c r="B14" t="s">
+      <c r="D14" t="s">
         <v>54</v>
       </c>
-      <c r="C14" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" t="s">
-        <v>33</v>
-      </c>
       <c r="E14" s="1">
-        <v>1.1726013</v>
+        <v>1750.380808</v>
       </c>
       <c r="F14" s="1">
-        <v>132776</v>
+        <v>282837.304</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" t="s">
+        <v>55</v>
+      </c>
+      <c r="B15" t="s">
         <v>56</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>57</v>
       </c>
-      <c r="C15" t="s">
-        <v>58</v>
-      </c>
       <c r="D15" t="s">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="E15" s="1">
-        <v>0.16857862</v>
+        <v>1714.497747</v>
       </c>
       <c r="F15" s="1">
-        <v>112791.21</v>
+        <v>28035</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B16" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" t="s">
         <v>60</v>
       </c>
-      <c r="B16" t="s">
-        <v>61</v>
-      </c>
-      <c r="C16" t="s">
-        <v>62</v>
-      </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E16" s="1">
-        <v>137.374110874</v>
+        <v>1455.59946</v>
       </c>
       <c r="F16" s="1">
-        <v>98462.00071001</v>
+        <v>276764</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" t="s">
         <v>63</v>
       </c>
-      <c r="B17" t="s">
+      <c r="D17" t="s">
         <v>64</v>
       </c>
-      <c r="C17" t="s">
-        <v>65</v>
-      </c>
-      <c r="D17" t="s">
-        <v>66</v>
-      </c>
       <c r="E17" s="1">
-        <v>258.192884</v>
+        <v>745.2152</v>
       </c>
       <c r="F17" s="1">
-        <v>70351.84</v>
+        <v>2682415.3</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" t="s">
+        <v>65</v>
+      </c>
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" t="s">
         <v>67</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>68</v>
       </c>
-      <c r="C18" t="s">
-        <v>69</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
       <c r="E18" s="1">
-        <v>328.4611488</v>
+        <v>552.6938761</v>
       </c>
       <c r="F18" s="1">
-        <v>48593.46263240699</v>
+        <v>166807.34</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" t="s">
+        <v>69</v>
+      </c>
+      <c r="B19" t="s">
         <v>70</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>71</v>
       </c>
-      <c r="C19" t="s">
-        <v>72</v>
-      </c>
       <c r="D19" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="E19" s="1">
-        <v>7843.502919093998</v>
+        <v>328.4611488</v>
       </c>
       <c r="F19" s="1">
-        <v>35155</v>
+        <v>48593.46263240699</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" t="s">
+        <v>72</v>
+      </c>
+      <c r="B20" t="s">
         <v>73</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>74</v>
       </c>
-      <c r="C20" t="s">
-        <v>75</v>
-      </c>
       <c r="D20" t="s">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="E20" s="1">
-        <v>0.009231945200000001</v>
+        <v>323.151</v>
       </c>
       <c r="F20" s="1">
-        <v>29930.89999999999</v>
+        <v>7630.83</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" t="s">
+        <v>75</v>
+      </c>
+      <c r="B21" t="s">
         <v>76</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>77</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>78</v>
       </c>
-      <c r="D21" t="s">
-        <v>33</v>
-      </c>
       <c r="E21" s="1">
-        <v>1992.54224118</v>
+        <v>258.192884</v>
       </c>
       <c r="F21" s="1">
-        <v>28260.55</v>
+        <v>70351.84</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1238,13 +1238,13 @@
         <v>81</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E22" s="1">
-        <v>1714.497747</v>
+        <v>137.374110874</v>
       </c>
       <c r="F22" s="1">
-        <v>28035</v>
+        <v>98462.00071001</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1258,27 +1258,27 @@
         <v>84</v>
       </c>
       <c r="D23" t="s">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="E23" s="1">
-        <v>4.31956</v>
+        <v>32.29878160000001</v>
       </c>
       <c r="F23" s="1">
-        <v>26386.97</v>
+        <v>1879081.3</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C24" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E24" s="1">
         <v>14.601081</v>
@@ -1289,22 +1289,22 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B25" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D25" t="s">
-        <v>91</v>
+        <v>29</v>
       </c>
       <c r="E25" s="1">
-        <v>1.191091</v>
+        <v>13.793487</v>
       </c>
       <c r="F25" s="1">
-        <v>23755.85</v>
+        <v>10227.5</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1318,13 +1318,13 @@
         <v>94</v>
       </c>
       <c r="D26" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E26" s="1">
-        <v>36569.9404315</v>
+        <v>12.89851</v>
       </c>
       <c r="F26" s="1">
-        <v>21076.455</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -1338,13 +1338,13 @@
         <v>97</v>
       </c>
       <c r="D27" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="E27" s="1">
-        <v>13.793487</v>
+        <v>8.55559</v>
       </c>
       <c r="F27" s="1">
-        <v>10227.5</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -1361,10 +1361,10 @@
         <v>101</v>
       </c>
       <c r="E28" s="1">
-        <v>3217.5016</v>
+        <v>4.95363</v>
       </c>
       <c r="F28" s="1">
-        <v>7799.26</v>
+        <v>4499</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -1378,13 +1378,13 @@
         <v>104</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="E29" s="1">
-        <v>323.151</v>
+        <v>4.31956</v>
       </c>
       <c r="F29" s="1">
-        <v>7630.83</v>
+        <v>26386.97</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -1398,133 +1398,133 @@
         <v>107</v>
       </c>
       <c r="D30" t="s">
-        <v>108</v>
+        <v>29</v>
       </c>
       <c r="E30" s="1">
-        <v>4.95363</v>
+        <v>3.600933003</v>
       </c>
       <c r="F30" s="1">
-        <v>4499</v>
+        <v>1784.29</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" t="s">
+        <v>108</v>
+      </c>
+      <c r="B31" t="s">
         <v>109</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>110</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>111</v>
       </c>
-      <c r="D31" t="s">
-        <v>112</v>
-      </c>
       <c r="E31" s="1">
-        <v>2285.37</v>
+        <v>2.944291</v>
       </c>
       <c r="F31" s="1">
-        <v>2221.03</v>
+        <v>1216</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" t="s">
+        <v>112</v>
+      </c>
+      <c r="B32" t="s">
         <v>113</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>114</v>
       </c>
-      <c r="C32" t="s">
-        <v>115</v>
-      </c>
       <c r="D32" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="E32" s="1">
-        <v>3.600933003</v>
+        <v>1.840197</v>
       </c>
       <c r="F32" s="1">
-        <v>1784.29</v>
+        <v>860.3</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" t="s">
+        <v>115</v>
+      </c>
+      <c r="B33" t="s">
         <v>116</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>117</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>118</v>
       </c>
-      <c r="D33" t="s">
-        <v>119</v>
-      </c>
       <c r="E33" s="1">
-        <v>0.613963</v>
+        <v>1.191091</v>
       </c>
       <c r="F33" s="1">
-        <v>1725</v>
+        <v>23755.85</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" t="s">
+        <v>119</v>
+      </c>
+      <c r="B34" t="s">
         <v>120</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>121</v>
       </c>
-      <c r="C34" t="s">
-        <v>122</v>
-      </c>
       <c r="D34" t="s">
-        <v>123</v>
+        <v>29</v>
       </c>
       <c r="E34" s="1">
-        <v>2.944291</v>
+        <v>1.1726013</v>
       </c>
       <c r="F34" s="1">
-        <v>1216</v>
+        <v>132776</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" t="s">
+        <v>122</v>
+      </c>
+      <c r="B35" t="s">
+        <v>123</v>
+      </c>
+      <c r="C35" t="s">
         <v>124</v>
       </c>
-      <c r="B35" t="s">
+      <c r="D35" t="s">
         <v>125</v>
       </c>
-      <c r="C35" t="s">
-        <v>126</v>
-      </c>
-      <c r="D35" t="s">
-        <v>91</v>
-      </c>
       <c r="E35" s="1">
-        <v>0.05379121</v>
+        <v>0.613963</v>
       </c>
       <c r="F35" s="1">
-        <v>1139</v>
+        <v>1725</v>
       </c>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" t="s">
+        <v>126</v>
+      </c>
+      <c r="B36" t="s">
         <v>127</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>128</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>129</v>
       </c>
-      <c r="D36" t="s">
-        <v>33</v>
-      </c>
       <c r="E36" s="1">
-        <v>1.840197</v>
+        <v>0.423747</v>
       </c>
       <c r="F36" s="1">
-        <v>860.3</v>
+        <v>0.2347</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1538,13 +1538,13 @@
         <v>132</v>
       </c>
       <c r="D37" t="s">
-        <v>33</v>
+        <v>68</v>
       </c>
       <c r="E37" s="1">
-        <v>0.36438</v>
+        <v>0.413115</v>
       </c>
       <c r="F37" s="1">
-        <v>111.2</v>
+        <v>0.316</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1558,33 +1558,33 @@
         <v>135</v>
       </c>
       <c r="D38" t="s">
-        <v>136</v>
+        <v>29</v>
       </c>
       <c r="E38" s="1">
-        <v>0.000140299</v>
+        <v>0.36438</v>
       </c>
       <c r="F38" s="1">
-        <v>54.06</v>
+        <v>111.2</v>
       </c>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" t="s">
+        <v>136</v>
+      </c>
+      <c r="B39" t="s">
         <v>137</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>138</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>139</v>
       </c>
-      <c r="D39" t="s">
-        <v>25</v>
-      </c>
       <c r="E39" s="1">
-        <v>8.55559</v>
+        <v>0.16857862</v>
       </c>
       <c r="F39" s="1">
-        <v>38.5</v>
+        <v>112791.21</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1598,13 +1598,13 @@
         <v>142</v>
       </c>
       <c r="D40" t="s">
-        <v>37</v>
+        <v>118</v>
       </c>
       <c r="E40" s="1">
-        <v>12.89851</v>
+        <v>0.05379121</v>
       </c>
       <c r="F40" s="1">
-        <v>0.99</v>
+        <v>1139</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1618,13 +1618,13 @@
         <v>145</v>
       </c>
       <c r="D41" t="s">
-        <v>52</v>
+        <v>68</v>
       </c>
       <c r="E41" s="1">
-        <v>0.413115</v>
+        <v>0.009231945200000001</v>
       </c>
       <c r="F41" s="1">
-        <v>0.316</v>
+        <v>29930.9</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1638,13 +1638,13 @@
         <v>148</v>
       </c>
       <c r="D42" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="E42" s="1">
-        <v>0.423747</v>
+        <v>0.000140299</v>
       </c>
       <c r="F42" s="1">
-        <v>0.2347</v>
+        <v>54.06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>